<commit_message>
Diapositivas del seminario final
</commit_message>
<xml_diff>
--- a/AVANCE DE ESCRITURA JUNIO/TABLAS Y FIGURAS BONITAS REV1.xlsx
+++ b/AVANCE DE ESCRITURA JUNIO/TABLAS Y FIGURAS BONITAS REV1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Angeal\Desktop\GNLPDA\AVANCE DE ESCRITURA JUNIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EB35DB5-6F20-491B-BF0F-B7EE07D9FE47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3046366-DB32-4D9D-85F1-09CD7AE6B2E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="77040" windowHeight="21120" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="77040" windowHeight="21120" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,12 @@
     <sheet name="Hoja5" sheetId="5" r:id="rId5"/>
     <sheet name="Hoja6" sheetId="6" r:id="rId6"/>
     <sheet name="Hoja7" sheetId="7" r:id="rId7"/>
+    <sheet name="Hoja8" sheetId="8" r:id="rId8"/>
+    <sheet name="Hoja9" sheetId="9" r:id="rId9"/>
+    <sheet name="Hoja10" sheetId="10" r:id="rId10"/>
+    <sheet name="Hoja11" sheetId="11" r:id="rId11"/>
+    <sheet name="Hoja12" sheetId="12" r:id="rId12"/>
+    <sheet name="Hoja13" sheetId="13" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Hoja7!$B$1:$B$89</definedName>
@@ -45,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="231">
   <si>
     <t>Dataset</t>
   </si>
@@ -525,12 +531,282 @@
   <si>
     <t>Referencias</t>
   </si>
+  <si>
+    <t>Autor y fecha</t>
+  </si>
+  <si>
+    <t>Yang et al. (2023); Araveeporn &amp; Banditvilai (2023)</t>
+  </si>
+  <si>
+    <t>Variantes Lineales (LDA Regularizado)</t>
+  </si>
+  <si>
+    <t>Agatra et al. (2025); Buhas et al. (2024)</t>
+  </si>
+  <si>
+    <t>Variantes Lineales (PCA-LDA)</t>
+  </si>
+  <si>
+    <t>Li et al. (2024); Shi &amp; Wu (2024)</t>
+  </si>
+  <si>
+    <t>Variantes Lineales (Trace-Ratio)</t>
+  </si>
+  <si>
+    <t>Medina et al. (2025); Briscik et al. (2023); Du et al. (2024)</t>
+  </si>
+  <si>
+    <t>Métodos Kernel (KPCA, KFDA)</t>
+  </si>
+  <si>
+    <t>Jalili et al. (2025); Remaki (2026)</t>
+  </si>
+  <si>
+    <t>Métodos Kernel (SVM)</t>
+  </si>
+  <si>
+    <t>Modelan fronteras altamente no lineales; exigen control estricto de parámetros para evitar sobreajuste.</t>
+  </si>
+  <si>
+    <t>Al-Milli et al. (2021); Wang et al. (2026)</t>
+  </si>
+  <si>
+    <t>Selección Evolutiva (Algoritmos Genéticos)</t>
+  </si>
+  <si>
+    <t>Wang et al. (2022); Manhrawy et al. (2026)</t>
+  </si>
+  <si>
+    <t>Métodos Híbridos</t>
+  </si>
+  <si>
+    <t>Medina et al. (2025)</t>
+  </si>
+  <si>
+    <t>Selección Evolutiva (GPDA)</t>
+  </si>
+  <si>
+    <t>Añaden regularización al modelo clásico para 
+estabilizar matrices en problemas de alta dimensionalidad.</t>
+  </si>
+  <si>
+    <t>Reducen la dimensionalidad en dos etapas 
+para eliminar redundancia antes de clasificar.</t>
+  </si>
+  <si>
+    <t>Optimizan directamente la relación de 
+dispersión interclase/intraclase para matrices singulares.</t>
+  </si>
+  <si>
+    <t>Emplean mapeos no lineales para
+ separar clases complejas, asumiendo pérdida de interpretabilidad.</t>
+  </si>
+  <si>
+    <t>Extraen subconjuntos de variables evadiendo óptimos
+ locales sin incurrir en costos computacionales prohibitivos.</t>
+  </si>
+  <si>
+    <t>Combinan filtrado estadístico inicial con 
+metaheurísticas para acelerar la selección de variables.</t>
+  </si>
+  <si>
+    <t>Maximizan la separabilidad evaluando proyecciones 
+directamente mediante el índice de silueta (sin invertir matrices).</t>
+  </si>
+  <si>
+    <t>Contibución</t>
+  </si>
+  <si>
+    <t>Apartado</t>
+  </si>
+  <si>
+    <t>Tabla 1: Estado del arte</t>
+  </si>
+  <si>
+    <t>X₁</t>
+  </si>
+  <si>
+    <t>X₂</t>
+  </si>
+  <si>
+    <t>X₁²</t>
+  </si>
+  <si>
+    <t>X₁X₂</t>
+  </si>
+  <si>
+    <t>X₂²</t>
+  </si>
+  <si>
+    <t>Componente</t>
+  </si>
+  <si>
+    <t>Configuración</t>
+  </si>
+  <si>
+    <t>Fit1 = Accuracy(cv5) – λ(n/N)
+Fit2 = Accuracy(cv5) – λ(n*/N*)</t>
+  </si>
+  <si>
+    <t>Selección de padres</t>
+  </si>
+  <si>
+    <t>Toreno binario</t>
+  </si>
+  <si>
+    <t>Oprador de cruza</t>
+  </si>
+  <si>
+    <t>Cruza de un solo punto</t>
+  </si>
+  <si>
+    <t>Operador de mutación</t>
+  </si>
+  <si>
+    <t>Mutación bit flip</t>
+  </si>
+  <si>
+    <t>Los mejores 2 de la generación pasan directo</t>
+  </si>
+  <si>
+    <t>Mecanismo de remplazo</t>
+  </si>
+  <si>
+    <t>Reemplazo generacional con elitismo</t>
+  </si>
+  <si>
+    <t>n_gen</t>
+  </si>
+  <si>
+    <t>popSize</t>
+  </si>
+  <si>
+    <t>p_cruza</t>
+  </si>
+  <si>
+    <t>p_mut</t>
+  </si>
+  <si>
+    <t>lambda</t>
+  </si>
+  <si>
+    <t>Descripción</t>
+  </si>
+  <si>
+    <t>Número de Generaciones</t>
+  </si>
+  <si>
+    <t>Probabilidad de Mutación</t>
+  </si>
+  <si>
+    <t>Parametro</t>
+  </si>
+  <si>
+    <t>Valores finales</t>
+  </si>
+  <si>
+    <t>Rango 
+min</t>
+  </si>
+  <si>
+    <t>Rango 
+max</t>
+  </si>
+  <si>
+    <t>Tamaño de
+ Población</t>
+  </si>
+  <si>
+    <t>Probabilidad de
+ Cruza</t>
+  </si>
+  <si>
+    <t>Factor de Penalización (λ)</t>
+  </si>
+  <si>
+    <t>Entero 
+(i)</t>
+  </si>
+  <si>
+    <t>Real 
+(r)</t>
+  </si>
+  <si>
+    <t>Tabla 4: Calibración de parametros</t>
+  </si>
+  <si>
+    <t>Función de aptitud</t>
+  </si>
+  <si>
+    <t>Tabla 3: Calibración de parametros</t>
+  </si>
+  <si>
+    <t>Binaria (Cromosomas de tamaño N)</t>
+  </si>
+  <si>
+    <t>Clasíficador</t>
+  </si>
+  <si>
+    <t>1.2.penguins_res_gnlpda.csv</t>
+  </si>
+  <si>
+    <t>1.3.pimadiabetes_res_gnlpda.csv</t>
+  </si>
+  <si>
+    <t>1.4.wines_res_gnlpda.csv</t>
+  </si>
+  <si>
+    <t>3.1.Cebolla3D_res_gnlpda.csv</t>
+  </si>
+  <si>
+    <t>3.2.Cebolla10D_res_gnlpda.csv</t>
+  </si>
+  <si>
+    <t>3.3.Cebolla20D_res_gnlpda.csv</t>
+  </si>
+  <si>
+    <t>4.1.CancerWisconsin_res_gnlpda.csv</t>
+  </si>
+  <si>
+    <t>4.2.Ionosphere_res_gnlpda.csv</t>
+  </si>
+  <si>
+    <t>5.4.indicadores2015_res_gnlpda.csv</t>
+  </si>
+  <si>
+    <t>5.5.indicadores2020_res_gnlpda.csv</t>
+  </si>
+  <si>
+    <t>Min</t>
+  </si>
+  <si>
+    <t>Max</t>
+  </si>
+  <si>
+    <t>Mediana</t>
+  </si>
+  <si>
+    <t>Media</t>
+  </si>
+  <si>
+    <t>Desv. Est.</t>
+  </si>
+  <si>
+    <t>Tiempo (D.E)</t>
+  </si>
+  <si>
+    <t>Tiempo 
+(Media)</t>
+  </si>
+  <si>
+    <t>Tabla 3: Resumen de rendimiento y tiempo de GNLPDA</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -593,8 +869,68 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -607,8 +943,38 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF9BBA58"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD0D7E8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDEE7D1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE9ECF4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEEF3EA"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -631,22 +997,137 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC4C7C5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFC4C7C5"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFC4C7C5"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFC4C7C5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFFFFFFF"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color rgb="FFFFFFFF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFFFFFFF"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="thick">
+        <color rgb="FFFFFFFF"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFFFFFFF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFFFFFFF"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFFFFFFF"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFFFFFFF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -655,11 +1136,98 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1219,6 +1787,1071 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4EE8590-F4BD-4325-A2C4-1CEA957237FA}">
+  <dimension ref="D3:K9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="3.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="4:11" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D3" s="17" t="s">
+        <v>174</v>
+      </c>
+      <c r="E3" s="17" t="s">
+        <v>175</v>
+      </c>
+      <c r="F3" s="18" t="s">
+        <v>176</v>
+      </c>
+      <c r="G3" s="18" t="s">
+        <v>177</v>
+      </c>
+      <c r="H3" s="18" t="s">
+        <v>178</v>
+      </c>
+      <c r="J3" s="18" t="s">
+        <v>176</v>
+      </c>
+      <c r="K3" s="18" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="4" spans="4:11" ht="24.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
+      <c r="H4" s="20"/>
+      <c r="J4" s="20"/>
+      <c r="K4" s="20"/>
+    </row>
+    <row r="5" spans="4:11" ht="24" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="22"/>
+      <c r="J5" s="22"/>
+      <c r="K5" s="22"/>
+    </row>
+    <row r="6" spans="4:11" ht="24" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D6" s="23"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="24"/>
+      <c r="H6" s="24"/>
+      <c r="J6" s="24"/>
+      <c r="K6" s="24"/>
+    </row>
+    <row r="7" spans="4:11" ht="24" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D7" s="21"/>
+      <c r="E7" s="21"/>
+      <c r="F7" s="22"/>
+      <c r="G7" s="22"/>
+      <c r="H7" s="22"/>
+      <c r="J7" s="22"/>
+      <c r="K7" s="22"/>
+    </row>
+    <row r="8" spans="4:11" ht="24" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D8" s="23"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="24"/>
+      <c r="G8" s="24"/>
+      <c r="H8" s="24"/>
+      <c r="J8" s="24"/>
+      <c r="K8" s="24"/>
+    </row>
+    <row r="9" spans="4:11" ht="24" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D9" s="21"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="22"/>
+      <c r="H9" s="22"/>
+      <c r="J9" s="22"/>
+      <c r="K9" s="22"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D65027B9-F002-4D22-8D70-8E6FEF0951ED}">
+  <dimension ref="C7:H16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="38.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="52.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="7" spans="3:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C7" s="11" t="s">
+        <v>210</v>
+      </c>
+      <c r="D7" s="11"/>
+      <c r="E7" s="32"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="32"/>
+      <c r="H7" s="32"/>
+    </row>
+    <row r="8" spans="3:8" ht="26.25" x14ac:dyDescent="0.25">
+      <c r="C8" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="9" spans="3:8" ht="48" x14ac:dyDescent="0.25">
+      <c r="C9" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="D9" s="33" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="10" spans="3:8" ht="46.5" x14ac:dyDescent="0.25">
+      <c r="C10" s="31" t="s">
+        <v>209</v>
+      </c>
+      <c r="D10" s="30" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="11" spans="3:8" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="C11" s="29" t="s">
+        <v>182</v>
+      </c>
+      <c r="D11" s="28" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="12" spans="3:8" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="C12" s="31" t="s">
+        <v>184</v>
+      </c>
+      <c r="D12" s="30" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="13" spans="3:8" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="C13" s="29" t="s">
+        <v>186</v>
+      </c>
+      <c r="D13" s="28" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="14" spans="3:8" ht="46.5" x14ac:dyDescent="0.25">
+      <c r="C14" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="28" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="15" spans="3:8" ht="46.5" x14ac:dyDescent="0.25">
+      <c r="C15" s="31" t="s">
+        <v>189</v>
+      </c>
+      <c r="D15" s="30" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="16" spans="3:8" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="C16" s="31" t="s">
+        <v>212</v>
+      </c>
+      <c r="D16" s="30" t="s">
+        <v>58</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C7:D7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB38107B-E033-4843-852C-AAABC10D6FE4}">
+  <dimension ref="D3:J27"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="14.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="4:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D3" s="11" t="s">
+        <v>208</v>
+      </c>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+    </row>
+    <row r="4" spans="4:9" ht="52.5" x14ac:dyDescent="0.25">
+      <c r="D4" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="5" spans="4:9" ht="46.5" x14ac:dyDescent="0.25">
+      <c r="D5" s="28" t="s">
+        <v>191</v>
+      </c>
+      <c r="E5" s="28" t="s">
+        <v>197</v>
+      </c>
+      <c r="F5" s="29" t="s">
+        <v>206</v>
+      </c>
+      <c r="G5" s="28">
+        <v>20</v>
+      </c>
+      <c r="H5" s="29">
+        <v>100</v>
+      </c>
+      <c r="I5" s="29">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="6" spans="4:9" ht="46.5" x14ac:dyDescent="0.25">
+      <c r="D6" s="30" t="s">
+        <v>192</v>
+      </c>
+      <c r="E6" s="30" t="s">
+        <v>203</v>
+      </c>
+      <c r="F6" s="31" t="s">
+        <v>206</v>
+      </c>
+      <c r="G6" s="30">
+        <v>20</v>
+      </c>
+      <c r="H6" s="31">
+        <v>100</v>
+      </c>
+      <c r="I6" s="31">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="7" spans="4:9" ht="46.5" x14ac:dyDescent="0.25">
+      <c r="D7" s="28" t="s">
+        <v>193</v>
+      </c>
+      <c r="E7" s="28" t="s">
+        <v>204</v>
+      </c>
+      <c r="F7" s="29" t="s">
+        <v>207</v>
+      </c>
+      <c r="G7" s="28">
+        <v>0.4</v>
+      </c>
+      <c r="H7" s="29">
+        <v>0.95</v>
+      </c>
+      <c r="I7" s="29">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="8" spans="4:9" ht="46.5" x14ac:dyDescent="0.25">
+      <c r="D8" s="30" t="s">
+        <v>194</v>
+      </c>
+      <c r="E8" s="30" t="s">
+        <v>198</v>
+      </c>
+      <c r="F8" s="31" t="s">
+        <v>207</v>
+      </c>
+      <c r="G8" s="30">
+        <v>0.05</v>
+      </c>
+      <c r="H8" s="31">
+        <v>0.2</v>
+      </c>
+      <c r="I8" s="31">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="9" spans="4:9" ht="46.5" x14ac:dyDescent="0.25">
+      <c r="D9" s="28" t="s">
+        <v>195</v>
+      </c>
+      <c r="E9" s="28" t="s">
+        <v>205</v>
+      </c>
+      <c r="F9" s="29" t="s">
+        <v>207</v>
+      </c>
+      <c r="G9" s="28">
+        <v>0.01</v>
+      </c>
+      <c r="H9" s="29">
+        <v>0.2</v>
+      </c>
+      <c r="I9" s="29">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="21" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="22" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F22" s="25"/>
+      <c r="G22" s="25"/>
+      <c r="H22" s="25"/>
+      <c r="I22" s="25"/>
+      <c r="J22" s="25"/>
+    </row>
+    <row r="23" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F23" s="26"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="26"/>
+      <c r="I23" s="26"/>
+      <c r="J23" s="26"/>
+    </row>
+    <row r="24" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F24" s="26"/>
+      <c r="G24" s="26"/>
+      <c r="H24" s="26"/>
+      <c r="I24" s="26"/>
+      <c r="J24" s="26"/>
+    </row>
+    <row r="25" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F25" s="26"/>
+      <c r="G25" s="26"/>
+      <c r="H25" s="26"/>
+      <c r="I25" s="26"/>
+      <c r="J25" s="26"/>
+    </row>
+    <row r="26" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F26" s="26"/>
+      <c r="G26" s="26"/>
+      <c r="H26" s="26"/>
+      <c r="I26" s="26"/>
+      <c r="J26" s="26"/>
+    </row>
+    <row r="27" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F27" s="26"/>
+      <c r="G27" s="26"/>
+      <c r="H27" s="26"/>
+      <c r="I27" s="26"/>
+      <c r="J27" s="26"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="D3:I3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{876F9CF3-7671-42E9-8B46-5CFD05DE74DC}">
+  <dimension ref="E10:AA37"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="5" max="5" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.42578125" customWidth="1"/>
+    <col min="13" max="13" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="10" spans="20:27" ht="30" x14ac:dyDescent="0.25">
+      <c r="T10" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="U10" s="27" t="s">
+        <v>223</v>
+      </c>
+      <c r="V10" s="27" t="s">
+        <v>224</v>
+      </c>
+      <c r="W10" s="27" t="s">
+        <v>225</v>
+      </c>
+      <c r="X10" s="27" t="s">
+        <v>226</v>
+      </c>
+      <c r="Y10" s="27" t="s">
+        <v>227</v>
+      </c>
+      <c r="Z10" s="34" t="s">
+        <v>229</v>
+      </c>
+      <c r="AA10" s="27" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="11" spans="20:27" x14ac:dyDescent="0.25">
+      <c r="T11" s="27" t="s">
+        <v>213</v>
+      </c>
+      <c r="U11" s="27">
+        <v>0.94</v>
+      </c>
+      <c r="V11" s="27">
+        <v>1</v>
+      </c>
+      <c r="W11" s="27">
+        <v>0.98</v>
+      </c>
+      <c r="X11" s="27">
+        <v>0.98</v>
+      </c>
+      <c r="Y11" s="27">
+        <v>0.01</v>
+      </c>
+      <c r="Z11" s="27">
+        <v>4.68</v>
+      </c>
+      <c r="AA11" s="27">
+        <v>5.68</v>
+      </c>
+    </row>
+    <row r="12" spans="20:27" x14ac:dyDescent="0.25">
+      <c r="T12" s="27" t="s">
+        <v>215</v>
+      </c>
+      <c r="U12" s="27">
+        <v>0.83</v>
+      </c>
+      <c r="V12" s="27">
+        <v>1</v>
+      </c>
+      <c r="W12" s="27">
+        <v>0.94</v>
+      </c>
+      <c r="X12" s="27">
+        <v>0.94</v>
+      </c>
+      <c r="Y12" s="27">
+        <v>0.04</v>
+      </c>
+      <c r="Z12" s="27">
+        <v>882.39</v>
+      </c>
+      <c r="AA12" s="27">
+        <v>441.21</v>
+      </c>
+    </row>
+    <row r="13" spans="20:27" x14ac:dyDescent="0.25">
+      <c r="T13" s="27" t="s">
+        <v>219</v>
+      </c>
+      <c r="U13" s="27">
+        <v>0.94</v>
+      </c>
+      <c r="V13" s="27">
+        <v>0.98</v>
+      </c>
+      <c r="W13" s="27">
+        <v>0.96</v>
+      </c>
+      <c r="X13" s="27">
+        <v>0.96</v>
+      </c>
+      <c r="Y13" s="27">
+        <v>0.01</v>
+      </c>
+      <c r="Z13" s="27">
+        <v>2496.7800000000002</v>
+      </c>
+      <c r="AA13" s="27">
+        <v>958.95</v>
+      </c>
+    </row>
+    <row r="14" spans="20:27" x14ac:dyDescent="0.25">
+      <c r="T14" s="27" t="s">
+        <v>220</v>
+      </c>
+      <c r="U14" s="27">
+        <v>0.84</v>
+      </c>
+      <c r="V14" s="27">
+        <v>0.95</v>
+      </c>
+      <c r="W14" s="27">
+        <v>0.89</v>
+      </c>
+      <c r="X14" s="27">
+        <v>0.89</v>
+      </c>
+      <c r="Y14" s="27">
+        <v>0.03</v>
+      </c>
+      <c r="Z14" s="27">
+        <v>3221.6</v>
+      </c>
+      <c r="AA14" s="27">
+        <v>1585.83</v>
+      </c>
+    </row>
+    <row r="15" spans="20:27" x14ac:dyDescent="0.25">
+      <c r="T15" s="27" t="s">
+        <v>216</v>
+      </c>
+      <c r="U15" s="27">
+        <v>0.93</v>
+      </c>
+      <c r="V15" s="27">
+        <v>0.99</v>
+      </c>
+      <c r="W15" s="27">
+        <v>0.97</v>
+      </c>
+      <c r="X15" s="27">
+        <v>0.97</v>
+      </c>
+      <c r="Y15" s="27">
+        <v>0.02</v>
+      </c>
+      <c r="Z15" s="27">
+        <v>3.83</v>
+      </c>
+      <c r="AA15" s="27">
+        <v>4.6500000000000004</v>
+      </c>
+    </row>
+    <row r="16" spans="20:27" x14ac:dyDescent="0.25">
+      <c r="T16" s="27" t="s">
+        <v>217</v>
+      </c>
+      <c r="U16" s="27">
+        <v>0.82</v>
+      </c>
+      <c r="V16" s="27">
+        <v>0.97</v>
+      </c>
+      <c r="W16" s="27">
+        <v>0.9</v>
+      </c>
+      <c r="X16" s="27">
+        <v>0.9</v>
+      </c>
+      <c r="Y16" s="27">
+        <v>0.03</v>
+      </c>
+      <c r="Z16" s="27">
+        <v>2238.17</v>
+      </c>
+      <c r="AA16" s="27">
+        <v>1102.28</v>
+      </c>
+    </row>
+    <row r="17" spans="5:27" x14ac:dyDescent="0.25">
+      <c r="T17" s="27" t="s">
+        <v>218</v>
+      </c>
+      <c r="U17" s="27">
+        <v>0.71</v>
+      </c>
+      <c r="V17" s="27">
+        <v>0.93</v>
+      </c>
+      <c r="W17" s="27">
+        <v>0.83</v>
+      </c>
+      <c r="X17" s="27">
+        <v>0.82</v>
+      </c>
+      <c r="Y17" s="27">
+        <v>0.05</v>
+      </c>
+      <c r="Z17" s="27">
+        <v>1772.73</v>
+      </c>
+      <c r="AA17" s="27">
+        <v>596.16</v>
+      </c>
+    </row>
+    <row r="18" spans="5:27" x14ac:dyDescent="0.25">
+      <c r="T18" s="27" t="s">
+        <v>214</v>
+      </c>
+      <c r="U18" s="27">
+        <v>0.72</v>
+      </c>
+      <c r="V18" s="27">
+        <v>0.81</v>
+      </c>
+      <c r="W18" s="27">
+        <v>0.77</v>
+      </c>
+      <c r="X18" s="27">
+        <v>0.77</v>
+      </c>
+      <c r="Y18" s="27">
+        <v>0.02</v>
+      </c>
+      <c r="Z18" s="27">
+        <v>515.97</v>
+      </c>
+      <c r="AA18" s="27">
+        <v>292.13</v>
+      </c>
+    </row>
+    <row r="19" spans="5:27" x14ac:dyDescent="0.25">
+      <c r="T19" s="27" t="s">
+        <v>221</v>
+      </c>
+      <c r="U19" s="27">
+        <v>0.9</v>
+      </c>
+      <c r="V19" s="27">
+        <v>0.94</v>
+      </c>
+      <c r="W19" s="27">
+        <v>0.92</v>
+      </c>
+      <c r="X19" s="27">
+        <v>0.92</v>
+      </c>
+      <c r="Y19" s="27">
+        <v>0.01</v>
+      </c>
+      <c r="Z19" s="27">
+        <v>1245.8399999999999</v>
+      </c>
+      <c r="AA19" s="27">
+        <v>321.24</v>
+      </c>
+    </row>
+    <row r="20" spans="5:27" x14ac:dyDescent="0.25">
+      <c r="T20" s="27" t="s">
+        <v>222</v>
+      </c>
+      <c r="U20" s="27">
+        <v>0.91</v>
+      </c>
+      <c r="V20" s="27">
+        <v>0.96</v>
+      </c>
+      <c r="W20" s="27">
+        <v>0.93</v>
+      </c>
+      <c r="X20" s="27">
+        <v>0.93</v>
+      </c>
+      <c r="Y20" s="27">
+        <v>0.01</v>
+      </c>
+      <c r="Z20" s="27">
+        <v>715.43</v>
+      </c>
+      <c r="AA20" s="27">
+        <v>39.82</v>
+      </c>
+    </row>
+    <row r="26" spans="5:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E26" s="36" t="s">
+        <v>230</v>
+      </c>
+      <c r="F26" s="37"/>
+      <c r="G26" s="37"/>
+      <c r="H26" s="37"/>
+      <c r="I26" s="37"/>
+      <c r="J26" s="37"/>
+      <c r="K26" s="37"/>
+      <c r="L26" s="37"/>
+      <c r="M26" s="37"/>
+    </row>
+    <row r="27" spans="5:27" ht="45" x14ac:dyDescent="0.25">
+      <c r="E27" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>224</v>
+      </c>
+      <c r="I27" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="J27" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="K27" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="L27" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="M27" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="N27" s="6"/>
+      <c r="O27" s="6"/>
+      <c r="P27" s="6"/>
+    </row>
+    <row r="28" spans="5:27" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="E28" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="F28" s="7">
+        <v>4</v>
+      </c>
+      <c r="G28" s="7">
+        <v>0.94</v>
+      </c>
+      <c r="H28" s="7">
+        <v>1</v>
+      </c>
+      <c r="I28" s="7">
+        <v>0.98</v>
+      </c>
+      <c r="J28" s="7">
+        <v>0.98</v>
+      </c>
+      <c r="K28" s="7">
+        <v>0.01</v>
+      </c>
+      <c r="L28" s="7">
+        <v>4.68</v>
+      </c>
+      <c r="M28" s="7">
+        <v>5.68</v>
+      </c>
+      <c r="N28" s="7"/>
+      <c r="O28" s="7"/>
+      <c r="P28" s="7"/>
+    </row>
+    <row r="29" spans="5:27" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="E29" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="F29" s="7">
+        <v>13</v>
+      </c>
+      <c r="G29" s="7">
+        <v>0.83</v>
+      </c>
+      <c r="H29" s="7">
+        <v>1</v>
+      </c>
+      <c r="I29" s="7">
+        <v>0.94</v>
+      </c>
+      <c r="J29" s="7">
+        <v>0.94</v>
+      </c>
+      <c r="K29" s="7">
+        <v>0.04</v>
+      </c>
+      <c r="L29" s="7">
+        <v>882.39</v>
+      </c>
+      <c r="M29" s="7">
+        <v>441.21</v>
+      </c>
+      <c r="N29" s="7"/>
+      <c r="O29" s="7"/>
+      <c r="P29" s="7"/>
+    </row>
+    <row r="30" spans="5:27" ht="67.5" x14ac:dyDescent="0.25">
+      <c r="E30" s="35" t="s">
+        <v>8</v>
+      </c>
+      <c r="F30" s="35">
+        <v>30</v>
+      </c>
+      <c r="G30" s="35">
+        <v>0.94</v>
+      </c>
+      <c r="H30" s="35">
+        <v>0.98</v>
+      </c>
+      <c r="I30" s="35">
+        <v>0.96</v>
+      </c>
+      <c r="J30" s="35">
+        <v>0.96</v>
+      </c>
+      <c r="K30" s="35">
+        <v>0.01</v>
+      </c>
+      <c r="L30" s="35">
+        <v>2496.7800000000002</v>
+      </c>
+      <c r="M30" s="35">
+        <v>958.95</v>
+      </c>
+      <c r="N30" s="7"/>
+      <c r="O30" s="7"/>
+      <c r="P30" s="7"/>
+    </row>
+    <row r="31" spans="5:27" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="E31" s="35" t="s">
+        <v>9</v>
+      </c>
+      <c r="F31" s="35">
+        <v>34</v>
+      </c>
+      <c r="G31" s="35">
+        <v>0.84</v>
+      </c>
+      <c r="H31" s="35">
+        <v>0.95</v>
+      </c>
+      <c r="I31" s="35">
+        <v>0.89</v>
+      </c>
+      <c r="J31" s="35">
+        <v>0.89</v>
+      </c>
+      <c r="K31" s="35">
+        <v>0.03</v>
+      </c>
+      <c r="L31" s="35">
+        <v>3221.6</v>
+      </c>
+      <c r="M31" s="35">
+        <v>1585.83</v>
+      </c>
+      <c r="N31" s="7"/>
+      <c r="O31" s="7"/>
+      <c r="P31" s="7"/>
+    </row>
+    <row r="32" spans="5:27" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="E32" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="F32" s="7">
+        <v>3</v>
+      </c>
+      <c r="G32" s="7">
+        <v>0.93</v>
+      </c>
+      <c r="H32" s="7">
+        <v>0.99</v>
+      </c>
+      <c r="I32" s="7">
+        <v>0.97</v>
+      </c>
+      <c r="J32" s="7">
+        <v>0.97</v>
+      </c>
+      <c r="K32" s="7">
+        <v>0.02</v>
+      </c>
+      <c r="L32" s="7">
+        <v>3.83</v>
+      </c>
+      <c r="M32" s="7">
+        <v>4.6500000000000004</v>
+      </c>
+      <c r="N32" s="7"/>
+      <c r="O32" s="7"/>
+      <c r="P32" s="7"/>
+    </row>
+    <row r="33" spans="5:16" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="E33" s="35" t="s">
+        <v>6</v>
+      </c>
+      <c r="F33" s="35">
+        <v>10</v>
+      </c>
+      <c r="G33" s="35">
+        <v>0.82</v>
+      </c>
+      <c r="H33" s="35">
+        <v>0.97</v>
+      </c>
+      <c r="I33" s="35">
+        <v>0.9</v>
+      </c>
+      <c r="J33" s="35">
+        <v>0.9</v>
+      </c>
+      <c r="K33" s="35">
+        <v>0.03</v>
+      </c>
+      <c r="L33" s="35">
+        <v>2238.17</v>
+      </c>
+      <c r="M33" s="35">
+        <v>1102.28</v>
+      </c>
+      <c r="N33" s="7"/>
+      <c r="O33" s="7"/>
+      <c r="P33" s="7"/>
+    </row>
+    <row r="34" spans="5:16" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="E34" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="F34" s="7">
+        <v>20</v>
+      </c>
+      <c r="G34" s="7">
+        <v>0.71</v>
+      </c>
+      <c r="H34" s="7">
+        <v>0.93</v>
+      </c>
+      <c r="I34" s="7">
+        <v>0.83</v>
+      </c>
+      <c r="J34" s="7">
+        <v>0.82</v>
+      </c>
+      <c r="K34" s="7">
+        <v>0.05</v>
+      </c>
+      <c r="L34" s="7">
+        <v>1772.73</v>
+      </c>
+      <c r="M34" s="7">
+        <v>596.16</v>
+      </c>
+      <c r="N34" s="7"/>
+      <c r="O34" s="7"/>
+      <c r="P34" s="7"/>
+    </row>
+    <row r="35" spans="5:16" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="E35" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="F35" s="7">
+        <v>8</v>
+      </c>
+      <c r="G35" s="7">
+        <v>0.72</v>
+      </c>
+      <c r="H35" s="7">
+        <v>0.81</v>
+      </c>
+      <c r="I35" s="7">
+        <v>0.77</v>
+      </c>
+      <c r="J35" s="7">
+        <v>0.77</v>
+      </c>
+      <c r="K35" s="7">
+        <v>0.02</v>
+      </c>
+      <c r="L35" s="7">
+        <v>515.97</v>
+      </c>
+      <c r="M35" s="7">
+        <v>292.13</v>
+      </c>
+      <c r="N35" s="7"/>
+      <c r="O35" s="7"/>
+      <c r="P35" s="7"/>
+    </row>
+    <row r="36" spans="5:16" ht="46.5" x14ac:dyDescent="0.25">
+      <c r="E36" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F36" s="7">
+        <v>12</v>
+      </c>
+      <c r="G36" s="7">
+        <v>0.9</v>
+      </c>
+      <c r="H36" s="7">
+        <v>0.94</v>
+      </c>
+      <c r="I36" s="7">
+        <v>0.92</v>
+      </c>
+      <c r="J36" s="7">
+        <v>0.92</v>
+      </c>
+      <c r="K36" s="7">
+        <v>0.01</v>
+      </c>
+      <c r="L36" s="7">
+        <v>1245.8399999999999</v>
+      </c>
+      <c r="M36" s="7">
+        <v>321.24</v>
+      </c>
+      <c r="N36" s="7"/>
+      <c r="O36" s="7"/>
+      <c r="P36" s="7"/>
+    </row>
+    <row r="37" spans="5:16" ht="46.5" x14ac:dyDescent="0.25">
+      <c r="E37" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F37" s="7">
+        <v>12</v>
+      </c>
+      <c r="G37" s="7">
+        <v>0.91</v>
+      </c>
+      <c r="H37" s="7">
+        <v>0.96</v>
+      </c>
+      <c r="I37" s="7">
+        <v>0.93</v>
+      </c>
+      <c r="J37" s="7">
+        <v>0.93</v>
+      </c>
+      <c r="K37" s="7">
+        <v>0.01</v>
+      </c>
+      <c r="L37" s="7">
+        <v>715.43</v>
+      </c>
+      <c r="M37" s="7">
+        <v>39.82</v>
+      </c>
+      <c r="N37" s="7"/>
+      <c r="O37" s="7"/>
+      <c r="P37" s="7"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="E26:M26"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05B65E1C-9B7D-42D0-B69B-48D45C721FC3}">
   <dimension ref="B4:F14"/>
@@ -2293,4 +3926,258 @@
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3754401-6611-4767-B988-2572F166D1D1}">
+  <dimension ref="C3:E13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="50.5703125" customWidth="1"/>
+    <col min="4" max="4" width="41.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="96" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="3:5" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="C3" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="D3" s="13"/>
+      <c r="E3" s="14"/>
+    </row>
+    <row r="4" spans="3:5" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="C4" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="5" spans="3:5" ht="46.5" x14ac:dyDescent="0.25">
+      <c r="C5" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="6" spans="3:5" ht="46.5" x14ac:dyDescent="0.25">
+      <c r="C6" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="D6" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="7" spans="3:5" ht="46.5" x14ac:dyDescent="0.25">
+      <c r="C7" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="D7" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="8" spans="3:5" ht="46.5" x14ac:dyDescent="0.25">
+      <c r="C8" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="D8" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="9" spans="3:5" ht="46.5" x14ac:dyDescent="0.25">
+      <c r="C9" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>156</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="10" spans="3:5" ht="46.5" x14ac:dyDescent="0.25">
+      <c r="C10" s="15" t="s">
+        <v>158</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="11" spans="3:5" ht="46.5" x14ac:dyDescent="0.25">
+      <c r="C11" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="12" spans="3:5" ht="47.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C12" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="D12" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="E12" s="15" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="13" spans="3:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C13" s="9"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C3:E3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F9C3E64-A213-4737-8650-48BC4F1F536F}">
+  <dimension ref="E3:G12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="5" max="5" width="54" customWidth="1"/>
+    <col min="6" max="6" width="36.42578125" customWidth="1"/>
+    <col min="7" max="7" width="79" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="5:7" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="E3" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="F3" s="13"/>
+      <c r="G3" s="14"/>
+    </row>
+    <row r="4" spans="5:7" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="E4" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="5" spans="5:7" ht="67.5" x14ac:dyDescent="0.25">
+      <c r="E5" s="16" t="s">
+        <v>147</v>
+      </c>
+      <c r="F5" s="16" t="s">
+        <v>148</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="6" spans="5:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="E6" s="16" t="s">
+        <v>149</v>
+      </c>
+      <c r="F6" s="16" t="s">
+        <v>150</v>
+      </c>
+      <c r="G6" s="16" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="7" spans="5:7" ht="67.5" x14ac:dyDescent="0.25">
+      <c r="E7" s="16" t="s">
+        <v>151</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>152</v>
+      </c>
+      <c r="G7" s="16" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="8" spans="5:7" ht="67.5" x14ac:dyDescent="0.25">
+      <c r="E8" s="16" t="s">
+        <v>153</v>
+      </c>
+      <c r="F8" s="16" t="s">
+        <v>154</v>
+      </c>
+      <c r="G8" s="16" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="9" spans="5:7" ht="67.5" x14ac:dyDescent="0.25">
+      <c r="E9" s="16" t="s">
+        <v>155</v>
+      </c>
+      <c r="F9" s="16" t="s">
+        <v>156</v>
+      </c>
+      <c r="G9" s="16" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="10" spans="5:7" ht="90" x14ac:dyDescent="0.25">
+      <c r="E10" s="16" t="s">
+        <v>158</v>
+      </c>
+      <c r="F10" s="16" t="s">
+        <v>159</v>
+      </c>
+      <c r="G10" s="16" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="11" spans="5:7" ht="67.5" x14ac:dyDescent="0.25">
+      <c r="E11" s="16" t="s">
+        <v>160</v>
+      </c>
+      <c r="F11" s="16" t="s">
+        <v>161</v>
+      </c>
+      <c r="G11" s="16" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="12" spans="5:7" ht="90" x14ac:dyDescent="0.25">
+      <c r="E12" s="16" t="s">
+        <v>162</v>
+      </c>
+      <c r="F12" s="16" t="s">
+        <v>163</v>
+      </c>
+      <c r="G12" s="16" t="s">
+        <v>170</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="E3:G3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>